<commit_message>
feat: complete week 3 backend milestone - accept orders, update order status, get technician jobs, and project documentation updates
</commit_message>
<xml_diff>
--- a/Sa2yanti_Gantt_Chart.xlsx
+++ b/Sa2yanti_Gantt_Chart.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Fainal Project\Sa2yanti\Sa2yanti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9077AB24-61E4-4125-88C4-FB077B483EDA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{445059D1-84A3-4909-BB03-167306955B10}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t>Week</t>
   </si>
@@ -636,7 +636,9 @@
       <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="6"/>
+      <c r="F3" s="6" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">

</xml_diff>